<commit_message>
feat(stage17): stabilize V29 and canonicalize database
</commit_message>
<xml_diff>
--- a/lithosite-Mine-Services/Database/Mine-Services-Database.xlsx
+++ b/lithosite-Mine-Services/Database/Mine-Services-Database.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="24975" windowHeight="10155" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Baseline" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_System" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Lists" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WorkFront" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operations" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maintenance" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issues" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plans" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HSE" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AuditLog" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="_Baseline" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="_System" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="_Lists" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Equipment" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="WorkFront" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Operations" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Maintenance" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Issues" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Plans" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="HSE" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="AuditLog" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="152511" fullCalcOnLoad="1"/>
@@ -964,7 +964,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>A.1</t>
+          <t>A.2</t>
         </is>
       </c>
     </row>
@@ -1650,7 +1650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1669,37 +1669,42 @@
           <t>equipment_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>unit_no</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>owner_type</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>owner_name</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>effective_from</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>effective_to</t>
         </is>

</xml_diff>